<commit_message>
Mise a jour du rapport PFE, des diagrammes UML/Gantt et de la soutenance.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/diagramme-gantt.xlsx
+++ b/diagramme-gantt.xlsx
@@ -518,29 +518,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="22" max="22"/>
+    <col width="7" customWidth="1" min="23" max="23"/>
+    <col width="7" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Diagramme de Gantt du projet — Stage du 6 mars au 6 juin 2026</t>
+          <t>Diagramme de Gantt du projet — Stage du 6 mars au 17 août 2026</t>
         </is>
       </c>
     </row>
@@ -607,12 +617,62 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Mai</t>
+          <t>Juin</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Juin</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Juin</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Juin</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Juin</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Juillet</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>Juillet</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>Juillet</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>Juillet</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Août</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>Août</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>Août</t>
         </is>
       </c>
     </row>
@@ -687,6 +747,56 @@
           <t>S14</t>
         </is>
       </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -697,28 +807,38 @@
       <c r="B4" s="4" t="inlineStr"/>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Conception UML (1 mois)</t>
+          <t>Conception UML (1 mois 1 sem.)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Réalisation (5 sem.)</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Réalisation (3 mois)</t>
+        </is>
+      </c>
       <c r="I4" s="6" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="6" t="inlineStr"/>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>Tests (2 sem.)</t>
-        </is>
-      </c>
-      <c r="M4" s="7" t="inlineStr"/>
-      <c r="N4" s="7" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="6" t="inlineStr"/>
+      <c r="N4" s="6" t="inlineStr"/>
+      <c r="O4" s="6" t="inlineStr"/>
+      <c r="P4" s="6" t="inlineStr"/>
+      <c r="Q4" s="6" t="inlineStr"/>
+      <c r="R4" s="6" t="inlineStr"/>
+      <c r="S4" s="6" t="inlineStr"/>
+      <c r="T4" s="6" t="inlineStr"/>
+      <c r="U4" s="7" t="inlineStr">
+        <is>
+          <t>Tests (3 sem.)</t>
+        </is>
+      </c>
+      <c r="V4" s="7" t="inlineStr"/>
+      <c r="W4" s="7" t="inlineStr"/>
+      <c r="X4" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -777,12 +897,12 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>1 mois</t>
+          <t>1 mois 1 sem.</t>
         </is>
       </c>
     </row>
@@ -794,17 +914,17 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>26/07/2026</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>5 sem.</t>
+          <t>3 mois</t>
         </is>
       </c>
     </row>
@@ -816,23 +936,23 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>06/06/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2 sem.</t>
+          <t>3 sem.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:X1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>

</xml_diff>